<commit_message>
fix: Show day-precision dates so fractional lags are traceable, black text, row heights
- Dates now display as "5 Aug 2022" instead of "Aug 2022" so readers
  can verify how lags like "5.6 months" are calculated
- Changed FONT_NOTES from gray (#666666) to black (#000000)
- Added explicit row heights (24pt title, 30pt headers) across all 9
  Excel tabs to prevent text clipping

https://claude.ai/code/session_01H7vorbotPWmSSpdBD4XXLP
</commit_message>
<xml_diff>
--- a/output/drug_approval_timelines.xlsx
+++ b/output/drug_approval_timelines.xlsx
@@ -41,7 +41,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="00000000"/>
       <sz val="8"/>
     </font>
     <font>
@@ -584,14 +584,14 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Enhertu (T-DXd) — 2L+ HER2+ mBC (DESTINY-Breast03)</t>
@@ -605,7 +605,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -665,7 +665,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Mar 2022</t>
+          <t>15 Mar 2022</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Sep 2021</t>
+          <t>19 Sep 2021</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>5 Aug 2022</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>24 Jan 2023</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>24 Jan 2023</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>24 Jan 2023</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>24 Jan 2023</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Jan 2023</t>
+          <t>24 Jan 2023</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>17 Feb 2023</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>1 Sep 2022</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>1 Sep 2022</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Oct 2023</t>
+          <t>25 Oct 2023</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>2 Feb 2023</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Feb 2023</t>
+          <t>22 Feb 2023</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Jul 2023</t>
+          <t>3 Jul 2023</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>28 Oct 2022</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Jun 2023</t>
+          <t>29 Jun 2023</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>15 Aug 2022</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1648,14 +1648,14 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Trodelvy (SG) — 3L+ mTNBC (ASCENT)</t>
@@ -1669,7 +1669,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Nov 2020</t>
+          <t>1 Nov 2020</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Sep 2020</t>
+          <t>19 Sep 2020</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Apr 2021</t>
+          <t>7 Apr 2021</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Nov 2021</t>
+          <t>10 Nov 2021</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Nov 2021</t>
+          <t>10 Nov 2021</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Nov 2021</t>
+          <t>10 Nov 2021</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Nov 2021</t>
+          <t>10 Nov 2021</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Dec 2021</t>
+          <t>15 Dec 2021</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Jul 2022</t>
+          <t>18 Jul 2022</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>May 2021</t>
+          <t>1 May 2021</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>May 2021</t>
+          <t>1 May 2021</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
+          <t>19 Oct 2021</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Jul 2023</t>
+          <t>12 Jul 2023</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>May 2022</t>
+          <t>19 May 2022</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Apr 2022</t>
+          <t>6 Apr 2022</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Aug 2022</t>
+          <t>9 Aug 2022</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>28 Oct 2022</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Oct 2022</t>
+          <t>1 Oct 2022</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Apr 2021</t>
+          <t>15 Apr 2021</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2715,14 +2715,14 @@
     <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Derived Lag Analysis (months from FDA approval)</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -3552,7 +3552,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Trodelvy (SG) — 1L mTNBC (BRCA-wt, PD-L1 CPS&lt;10) (ASCENT-03)</t>
@@ -3566,7 +3566,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -3631,17 +3631,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Jul 2028</t>
+          <t>1 Jul 2028</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Jul 2028</t>
+          <t>1 Jul 2028</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Jul 2028</t>
+          <t>1 Jul 2028</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -3678,17 +3678,17 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>1 Dec 2025</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>1 Dec 2025</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>1 Dec 2025</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -3725,17 +3725,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -3772,17 +3772,17 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -3819,17 +3819,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -3866,17 +3866,17 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -3913,17 +3913,17 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -3960,17 +3960,17 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>2 Apr 2027</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>11 May 2027</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -4007,17 +4007,17 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>29 Jul 2027</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>13 Dec 2027</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -4054,17 +4054,17 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -4101,17 +4101,17 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -4148,17 +4148,17 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>16 Nov 2025</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -4195,17 +4195,17 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>16 Nov 2025</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -4242,17 +4242,17 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>16 Nov 2025</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -4289,17 +4289,17 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>16 Nov 2025</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -4336,17 +4336,17 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>16 Nov 2025</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>14 Mar 2027</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -4383,17 +4383,17 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>22 Nov 2027</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>May 2028</t>
+          <t>29 May 2028</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>Dec 2028</t>
+          <t>6 Dec 2028</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -4430,17 +4430,17 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>27 Feb 2027</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>23 Jun 2027</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>13 Oct 2027</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -4477,17 +4477,17 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>11 Jun 2027</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>1 Sep 2027</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -4524,17 +4524,17 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>29 Jul 2027</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>16 Oct 2027</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>4 Jan 2028</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -4571,17 +4571,17 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>25 Nov 2026</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>26 Jul 2027</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>23 Mar 2028</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -4618,17 +4618,17 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>26 Jul 2027</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>10 Nov 2027</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>24 Feb 2028</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -4665,17 +4665,17 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -4712,17 +4712,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
@@ -4759,17 +4759,17 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>22 Nov 2027</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>May 2028</t>
+          <t>29 May 2028</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Dec 2028</t>
+          <t>6 Dec 2028</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
@@ -4806,17 +4806,17 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>11 Jun 2027</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>1 Sep 2027</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -4853,17 +4853,17 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>18 Feb 2027</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
@@ -4900,17 +4900,17 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>29 Jul 2027</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>16 Oct 2027</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>4 Jan 2028</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
@@ -4947,17 +4947,17 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>25 Nov 2026</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>26 Jul 2027</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>23 Mar 2028</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -4994,17 +4994,17 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>26 Jul 2027</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>10 Nov 2027</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>24 Feb 2028</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
@@ -5058,7 +5058,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Trodelvy (SG) + Keytruda — 1L mTNBC (PD-L1 CPS&gt;=10) (ASCENT-04)</t>
@@ -5072,7 +5072,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -5137,17 +5137,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>1 Feb 2027</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>1 Feb 2027</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>1 Feb 2027</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -5184,17 +5184,17 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>21 Jan 2026</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>21 Jan 2026</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>21 Jan 2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -5231,17 +5231,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Oct 2026</t>
+          <t>1 Oct 2026</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -5278,17 +5278,17 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>10 Apr 2027</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>5 May 2027</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -5325,17 +5325,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>10 Apr 2027</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>5 May 2027</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -5372,17 +5372,17 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>10 Apr 2027</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>5 May 2027</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -5419,17 +5419,17 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>10 Apr 2027</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>5 May 2027</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -5466,17 +5466,17 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>2 May 2027</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>10 Jun 2027</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -5513,17 +5513,17 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>28 Aug 2027</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Jan 2028</t>
+          <t>12 Jan 2028</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -5560,17 +5560,17 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -5607,17 +5607,17 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -5650,17 +5650,17 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>16 Dec 2025</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -5697,17 +5697,17 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>16 Dec 2025</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -5744,17 +5744,17 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>16 Dec 2025</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -5791,17 +5791,17 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>16 Dec 2025</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -5838,17 +5838,17 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>16 Dec 2025</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>13 Apr 2027</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -5885,17 +5885,17 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>22 Dec 2027</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Jun 2028</t>
+          <t>28 Jun 2028</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>5 Jan 2029</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -5932,17 +5932,17 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>29 Mar 2027</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>23 Jul 2027</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>12 Nov 2027</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -5979,17 +5979,17 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>19 Apr 2027</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>11 Jul 2027</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>1 Oct 2027</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -6026,17 +6026,17 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>28 Aug 2027</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>15 Nov 2027</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>3 Feb 2028</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -6073,17 +6073,17 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>25 Aug 2027</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>22 Apr 2028</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -6120,17 +6120,17 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>25 Aug 2027</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>10 Dec 2027</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>25 Mar 2028</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -6167,17 +6167,17 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -6214,17 +6214,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>1 Nov 2026</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
@@ -6261,17 +6261,17 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>22 Dec 2027</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>Jun 2028</t>
+          <t>28 Jun 2028</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>5 Jan 2029</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
@@ -6308,17 +6308,17 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>19 Apr 2027</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>11 Jul 2027</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>1 Oct 2027</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -6355,17 +6355,17 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>20 Mar 2027</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>10 Apr 2027</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>May 2027</t>
+          <t>5 May 2027</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>28 Aug 2027</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>15 Nov 2027</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>3 Feb 2028</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
@@ -6449,17 +6449,17 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>25 Aug 2027</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Apr 2028</t>
+          <t>22 Apr 2028</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -6496,17 +6496,17 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>25 Aug 2027</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>10 Dec 2027</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>25 Mar 2028</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
@@ -6561,7 +6561,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dato-DXd (Datroway) — 1L mTNBC (BRCA-wt, PD-L1 CPS&lt;10) (TROPION-Breast02)</t>
@@ -6575,7 +6575,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -6640,17 +6640,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Mar 2025</t>
+          <t>1 Mar 2025</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Mar 2025</t>
+          <t>1 Mar 2025</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Mar 2025</t>
+          <t>1 Mar 2025</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -6687,17 +6687,17 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Jun 2025</t>
+          <t>1 Jun 2025</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Jun 2025</t>
+          <t>1 Jun 2025</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Jun 2025</t>
+          <t>1 Jun 2025</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -6734,17 +6734,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Jun 2026</t>
+          <t>1 Jun 2026</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Jun 2026</t>
+          <t>1 Jun 2026</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Jun 2026</t>
+          <t>1 Jun 2026</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -6781,17 +6781,17 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -6824,17 +6824,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -6871,17 +6871,17 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -6914,17 +6914,17 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -6957,17 +6957,17 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>18 Nov 2026</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>31 Dec 2026</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Feb 2027</t>
+          <t>8 Feb 2027</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -7004,17 +7004,17 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>28 Apr 2027</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Sep 2027</t>
+          <t>12 Sep 2027</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -7051,17 +7051,17 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -7098,17 +7098,17 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>15 Jan 2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -7141,17 +7141,17 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>16 Aug 2025</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -7188,17 +7188,17 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>16 Aug 2025</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -7235,17 +7235,17 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>16 Aug 2025</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -7282,17 +7282,17 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>16 Aug 2025</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -7329,17 +7329,17 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Aug 2025</t>
+          <t>16 Aug 2025</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Apr 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -7376,17 +7376,17 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>22 Aug 2027</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>27 Feb 2028</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>Sep 2028</t>
+          <t>5 Sep 2028</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -7423,17 +7423,17 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Nov 2026</t>
+          <t>27 Nov 2026</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>23 Mar 2027</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>13 Jul 2027</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -7470,17 +7470,17 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>18 Dec 2026</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>1 Jun 2027</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -7517,17 +7517,17 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>28 Apr 2027</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>16 Jul 2027</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>4 Oct 2027</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -7564,17 +7564,17 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>25 Apr 2027</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>22 Dec 2027</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -7611,17 +7611,17 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>25 Apr 2027</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>10 Aug 2027</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>24 Nov 2027</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -7658,17 +7658,17 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -7705,17 +7705,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>1 Jul 2026</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
@@ -7752,17 +7752,17 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>22 Aug 2027</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>Feb 2028</t>
+          <t>27 Feb 2028</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Sep 2028</t>
+          <t>5 Sep 2028</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
@@ -7799,17 +7799,17 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>18 Dec 2026</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Mar 2027</t>
+          <t>11 Mar 2027</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Jun 2027</t>
+          <t>1 Jun 2027</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -7846,17 +7846,17 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Sep 2026</t>
+          <t>1 Sep 2026</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Dec 2026</t>
+          <t>12 Dec 2026</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
@@ -7893,17 +7893,17 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>28 Apr 2027</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>16 Jul 2027</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Oct 2027</t>
+          <t>4 Oct 2027</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
@@ -7940,17 +7940,17 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>25 Aug 2026</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>25 Apr 2027</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Dec 2027</t>
+          <t>22 Dec 2027</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -7987,17 +7987,17 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Apr 2027</t>
+          <t>25 Apr 2027</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Aug 2027</t>
+          <t>10 Aug 2027</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Nov 2027</t>
+          <t>24 Nov 2027</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
@@ -8055,7 +8055,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dato-DXd (Datroway) +/- Durvalumab — 1L mTNBC (PD-L1 CPS&gt;=10) (TROPION-Breast05)</t>
@@ -8069,7 +8069,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
@@ -8134,17 +8134,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>28 Jul 2027</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>28 Jul 2027</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Jul 2027</t>
+          <t>28 Jul 2027</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -8181,17 +8181,17 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>1 Mar 2028</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>1 Mar 2028</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>1 Mar 2028</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -8228,17 +8228,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>1 Jan 2029</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>1 Jan 2029</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>1 Jan 2029</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -8275,17 +8275,17 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>11 Jul 2029</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>5 Aug 2029</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -8322,17 +8322,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>11 Jul 2029</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>5 Aug 2029</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
@@ -8369,17 +8369,17 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>11 Jul 2029</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>5 Aug 2029</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -8416,17 +8416,17 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>11 Jul 2029</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>5 Aug 2029</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -8463,17 +8463,17 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>2 Aug 2029</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Sep 2029</t>
+          <t>10 Sep 2029</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -8510,17 +8510,17 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>28 Nov 2029</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Apr 2030</t>
+          <t>14 Apr 2030</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -8557,17 +8557,17 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>25 Jan 2029</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>28 Jan 2029</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>28 Jan 2029</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -8604,17 +8604,17 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>25 Jan 2029</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>28 Jan 2029</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Jan 2029</t>
+          <t>28 Jan 2029</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -8651,17 +8651,17 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>18 Mar 2028</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Nov 2028</t>
+          <t>17 Nov 2028</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -8698,17 +8698,17 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>18 Mar 2028</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Nov 2028</t>
+          <t>17 Nov 2028</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -8745,17 +8745,17 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>18 Mar 2028</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Nov 2028</t>
+          <t>17 Nov 2028</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -8792,17 +8792,17 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>18 Mar 2028</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Nov 2028</t>
+          <t>17 Nov 2028</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -8839,17 +8839,17 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Mar 2028</t>
+          <t>18 Mar 2028</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Nov 2028</t>
+          <t>17 Nov 2028</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>14 Jul 2029</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -8886,17 +8886,17 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Mar 2030</t>
+          <t>24 Mar 2030</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Sep 2030</t>
+          <t>29 Sep 2030</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>Apr 2031</t>
+          <t>8 Apr 2031</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -8933,17 +8933,17 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>29 Jun 2029</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Oct 2029</t>
+          <t>23 Oct 2029</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>Feb 2030</t>
+          <t>12 Feb 2030</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -8980,17 +8980,17 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>20 Jul 2029</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Oct 2029</t>
+          <t>11 Oct 2029</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Jan 2030</t>
+          <t>1 Jan 2030</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -9027,17 +9027,17 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>28 Nov 2029</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>Feb 2030</t>
+          <t>15 Feb 2030</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>May 2030</t>
+          <t>6 May 2030</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -9074,17 +9074,17 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Mar 2029</t>
+          <t>27 Mar 2029</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>25 Nov 2029</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Jul 2030</t>
+          <t>24 Jul 2030</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -9121,17 +9121,17 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>25 Nov 2029</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Mar 2030</t>
+          <t>12 Mar 2030</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Jun 2030</t>
+          <t>26 Jun 2030</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -9168,17 +9168,17 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
@@ -9211,17 +9211,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Feb 2029</t>
+          <t>1 Feb 2029</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
@@ -9258,17 +9258,17 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Mar 2030</t>
+          <t>24 Mar 2030</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>Sep 2030</t>
+          <t>29 Sep 2030</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Apr 2031</t>
+          <t>8 Apr 2031</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
@@ -9305,17 +9305,17 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>20 Jul 2029</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Oct 2029</t>
+          <t>11 Oct 2029</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Jan 2030</t>
+          <t>1 Jan 2030</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
@@ -9352,17 +9352,17 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Jun 2029</t>
+          <t>20 Jun 2029</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Jul 2029</t>
+          <t>11 Jul 2029</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Aug 2029</t>
+          <t>5 Aug 2029</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
@@ -9399,17 +9399,17 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>28 Nov 2029</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Feb 2030</t>
+          <t>15 Feb 2030</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>May 2030</t>
+          <t>6 May 2030</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
@@ -9446,17 +9446,17 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Mar 2029</t>
+          <t>27 Mar 2029</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>25 Nov 2029</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Jul 2030</t>
+          <t>24 Jul 2030</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -9493,17 +9493,17 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Nov 2029</t>
+          <t>25 Nov 2029</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>Mar 2030</t>
+          <t>12 Mar 2030</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Jun 2030</t>
+          <t>26 Jun 2030</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
@@ -9552,14 +9552,14 @@
     <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Assumptions &amp; Data Gaps Log</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ID</t>
@@ -10769,7 +10769,7 @@
     <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Corcept Phase 3 Enrollment Implications</t>
@@ -10805,7 +10805,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Geography</t>

</xml_diff>